<commit_message>
Fase 2 replicada en la instancia usac-g3 (Odoo 20)
El script 01 instala CRM, Inventario y Compras. Los scripts 05 y 10
buscan el NIT con y sin guion, porque Odoo 20 lo guarda sin guion.
Productos.xlsx apunta a las imágenes de la nueva instancia. El Manual
Técnico y el zip de entrega tienen la URL, la base, la versión y la
fecha de entrega actualizadas.
</commit_message>
<xml_diff>
--- a/Productos.xlsx
+++ b/Productos.xlsx
@@ -1038,7 +1038,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/186/UJ-P01.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/637/UJ-P01.jpg</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/187/UJ-P02.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/638/UJ-P02.jpg</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/188/UJ-P03.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/639/UJ-P03.jpg</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/189/UJ-P04.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/640/UJ-P04.jpg</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/190/UJ-P05.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/641/UJ-P05.jpg</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/191/UJ-P06.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/642/UJ-P06.jpg</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/192/UJ-P07.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/643/UJ-P07.jpg</t>
         </is>
       </c>
     </row>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/193/UJ-P08.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/644/UJ-P08.jpg</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/194/UJ-P09.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/645/UJ-P09.jpg</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1407,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/195/UJ-P10.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/646/UJ-P10.jpg</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/196/UJ-P11.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/647/UJ-P11.jpg</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/197/UJ-P12.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/648/UJ-P12.jpg</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/198/UJ-P13.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/649/UJ-P13.jpg</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/199/UJ-P14.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/650/UJ-P14.jpg</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/200/UJ-P15.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/651/UJ-P15.jpg</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/201/UJ-P16.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/652/UJ-P16.jpg</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/202/UJ-P17.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/653/UJ-P17.jpg</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/203/UJ-P18.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/654/UJ-P18.jpg</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/204/UJ-P19.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/655/UJ-P19.jpg</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>https://usac.odoo.com/web/image/205/UJ-P20.jpg</t>
+          <t>https://usac-g3.odoo.com/web/image/656/UJ-P20.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>